<commit_message>
Reconferência do checador: 12 de 13 OK, falta a Res. 4.881 nas fontes da página
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LEmDYK8ehtpTRFSK7FMy6P
</commit_message>
<xml_diff>
--- a/produtos/chefoes-do-cartao/bonus/Placar-dos-Chefoes.xlsx
+++ b/produtos/chefoes-do-cartao/bonus/Placar-dos-Chefoes.xlsx
@@ -1763,7 +1763,7 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="3" customWidth="1" min="15" max="15"/>
@@ -2675,24 +2675,25 @@
       <c r="O26" s="1" t="n"/>
     </row>
     <row r="27" ht="19" customHeight="1">
-      <c r="A27" s="54" t="n">
-        <v>1</v>
+      <c r="A27" s="54">
+        <f>IF(COUNT($M$11:$M$20)&gt;=1,1,"")</f>
+        <v/>
       </c>
       <c r="B27" s="55">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($A27,$M$11:$M$20,0)),"")</f>
+        <f>IF($A27="","",IFERROR(INDEX($B$11:$B$20,MATCH($A27,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="C27" s="55">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($A27,$M$11:$M$20,0)),"")</f>
+        <f>IF($A27="","",IFERROR(INDEX($D$11:$D$20,MATCH($A27,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="D27" s="56" t="n"/>
       <c r="E27" s="57">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($A27,$M$11:$M$20,0)),"")</f>
+        <f>IF($A27="","",IFERROR(INDEX($E$11:$E$20,MATCH($A27,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="F27" s="58">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($A27,$M$11:$M$20,0)),"")</f>
+        <f>IF($A27="","",IFERROR(INDEX($H$11:$H$20,MATCH($A27,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="G27" s="59" t="inlineStr">
@@ -2700,430 +2701,449 @@
           <t>← ALVO</t>
         </is>
       </c>
-      <c r="H27" s="54" t="n">
-        <v>1</v>
+      <c r="H27" s="54">
+        <f>IF(COUNT($N$11:$N$20)&gt;=1,1,"")</f>
+        <v/>
       </c>
       <c r="I27" s="55">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($H27,$N$11:$N$20,0)),"")</f>
+        <f>IF($H27="","",IFERROR(INDEX($B$11:$B$20,MATCH($H27,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="J27" s="56" t="n"/>
       <c r="K27" s="56" t="n"/>
       <c r="L27" s="55">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($H27,$N$11:$N$20,0)),"")</f>
+        <f>IF($H27="","",IFERROR(INDEX($D$11:$D$20,MATCH($H27,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="M27" s="57">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($H27,$N$11:$N$20,0)),"")</f>
+        <f>IF($H27="","",IFERROR(INDEX($E$11:$E$20,MATCH($H27,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="N27" s="58">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($H27,$N$11:$N$20,0)),"")</f>
+        <f>IF($H27="","",IFERROR(INDEX($H$11:$H$20,MATCH($H27,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="O27" s="1" t="n"/>
     </row>
     <row r="28" ht="19" customHeight="1">
-      <c r="A28" s="45" t="n">
-        <v>2</v>
+      <c r="A28" s="45">
+        <f>IF(COUNT($M$11:$M$20)&gt;=2,2,"")</f>
+        <v/>
       </c>
       <c r="B28" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($A28,$M$11:$M$20,0)),"")</f>
+        <f>IF($A28="","",IFERROR(INDEX($B$11:$B$20,MATCH($A28,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="C28" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($A28,$M$11:$M$20,0)),"")</f>
+        <f>IF($A28="","",IFERROR(INDEX($D$11:$D$20,MATCH($A28,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="D28" s="60" t="n"/>
       <c r="E28" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($A28,$M$11:$M$20,0)),"")</f>
+        <f>IF($A28="","",IFERROR(INDEX($E$11:$E$20,MATCH($A28,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="F28" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($A28,$M$11:$M$20,0)),"")</f>
+        <f>IF($A28="","",IFERROR(INDEX($H$11:$H$20,MATCH($A28,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="G28" s="1" t="n"/>
-      <c r="H28" s="45" t="n">
-        <v>2</v>
+      <c r="H28" s="45">
+        <f>IF(COUNT($N$11:$N$20)&gt;=2,2,"")</f>
+        <v/>
       </c>
       <c r="I28" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($H28,$N$11:$N$20,0)),"")</f>
+        <f>IF($H28="","",IFERROR(INDEX($B$11:$B$20,MATCH($H28,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="J28" s="60" t="n"/>
       <c r="K28" s="60" t="n"/>
       <c r="L28" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($H28,$N$11:$N$20,0)),"")</f>
+        <f>IF($H28="","",IFERROR(INDEX($D$11:$D$20,MATCH($H28,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="M28" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($H28,$N$11:$N$20,0)),"")</f>
+        <f>IF($H28="","",IFERROR(INDEX($E$11:$E$20,MATCH($H28,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="N28" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($H28,$N$11:$N$20,0)),"")</f>
+        <f>IF($H28="","",IFERROR(INDEX($H$11:$H$20,MATCH($H28,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="O28" s="1" t="n"/>
     </row>
     <row r="29" ht="19" customHeight="1">
-      <c r="A29" s="45" t="n">
-        <v>3</v>
+      <c r="A29" s="45">
+        <f>IF(COUNT($M$11:$M$20)&gt;=3,3,"")</f>
+        <v/>
       </c>
       <c r="B29" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($A29,$M$11:$M$20,0)),"")</f>
+        <f>IF($A29="","",IFERROR(INDEX($B$11:$B$20,MATCH($A29,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="C29" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($A29,$M$11:$M$20,0)),"")</f>
+        <f>IF($A29="","",IFERROR(INDEX($D$11:$D$20,MATCH($A29,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="D29" s="60" t="n"/>
       <c r="E29" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($A29,$M$11:$M$20,0)),"")</f>
+        <f>IF($A29="","",IFERROR(INDEX($E$11:$E$20,MATCH($A29,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="F29" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($A29,$M$11:$M$20,0)),"")</f>
+        <f>IF($A29="","",IFERROR(INDEX($H$11:$H$20,MATCH($A29,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="G29" s="1" t="n"/>
-      <c r="H29" s="45" t="n">
-        <v>3</v>
+      <c r="H29" s="45">
+        <f>IF(COUNT($N$11:$N$20)&gt;=3,3,"")</f>
+        <v/>
       </c>
       <c r="I29" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($H29,$N$11:$N$20,0)),"")</f>
+        <f>IF($H29="","",IFERROR(INDEX($B$11:$B$20,MATCH($H29,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="J29" s="60" t="n"/>
       <c r="K29" s="60" t="n"/>
       <c r="L29" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($H29,$N$11:$N$20,0)),"")</f>
+        <f>IF($H29="","",IFERROR(INDEX($D$11:$D$20,MATCH($H29,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="M29" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($H29,$N$11:$N$20,0)),"")</f>
+        <f>IF($H29="","",IFERROR(INDEX($E$11:$E$20,MATCH($H29,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="N29" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($H29,$N$11:$N$20,0)),"")</f>
+        <f>IF($H29="","",IFERROR(INDEX($H$11:$H$20,MATCH($H29,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="O29" s="1" t="n"/>
     </row>
     <row r="30" ht="19" customHeight="1">
-      <c r="A30" s="45" t="n">
-        <v>4</v>
+      <c r="A30" s="45">
+        <f>IF(COUNT($M$11:$M$20)&gt;=4,4,"")</f>
+        <v/>
       </c>
       <c r="B30" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($A30,$M$11:$M$20,0)),"")</f>
+        <f>IF($A30="","",IFERROR(INDEX($B$11:$B$20,MATCH($A30,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="C30" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($A30,$M$11:$M$20,0)),"")</f>
+        <f>IF($A30="","",IFERROR(INDEX($D$11:$D$20,MATCH($A30,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="D30" s="60" t="n"/>
       <c r="E30" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($A30,$M$11:$M$20,0)),"")</f>
+        <f>IF($A30="","",IFERROR(INDEX($E$11:$E$20,MATCH($A30,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="F30" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($A30,$M$11:$M$20,0)),"")</f>
+        <f>IF($A30="","",IFERROR(INDEX($H$11:$H$20,MATCH($A30,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="G30" s="1" t="n"/>
-      <c r="H30" s="45" t="n">
-        <v>4</v>
+      <c r="H30" s="45">
+        <f>IF(COUNT($N$11:$N$20)&gt;=4,4,"")</f>
+        <v/>
       </c>
       <c r="I30" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($H30,$N$11:$N$20,0)),"")</f>
+        <f>IF($H30="","",IFERROR(INDEX($B$11:$B$20,MATCH($H30,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="J30" s="60" t="n"/>
       <c r="K30" s="60" t="n"/>
       <c r="L30" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($H30,$N$11:$N$20,0)),"")</f>
+        <f>IF($H30="","",IFERROR(INDEX($D$11:$D$20,MATCH($H30,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="M30" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($H30,$N$11:$N$20,0)),"")</f>
+        <f>IF($H30="","",IFERROR(INDEX($E$11:$E$20,MATCH($H30,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="N30" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($H30,$N$11:$N$20,0)),"")</f>
+        <f>IF($H30="","",IFERROR(INDEX($H$11:$H$20,MATCH($H30,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="O30" s="1" t="n"/>
     </row>
     <row r="31" ht="19" customHeight="1">
-      <c r="A31" s="45" t="n">
-        <v>5</v>
+      <c r="A31" s="45">
+        <f>IF(COUNT($M$11:$M$20)&gt;=5,5,"")</f>
+        <v/>
       </c>
       <c r="B31" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($A31,$M$11:$M$20,0)),"")</f>
+        <f>IF($A31="","",IFERROR(INDEX($B$11:$B$20,MATCH($A31,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="C31" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($A31,$M$11:$M$20,0)),"")</f>
+        <f>IF($A31="","",IFERROR(INDEX($D$11:$D$20,MATCH($A31,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="D31" s="60" t="n"/>
       <c r="E31" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($A31,$M$11:$M$20,0)),"")</f>
+        <f>IF($A31="","",IFERROR(INDEX($E$11:$E$20,MATCH($A31,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="F31" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($A31,$M$11:$M$20,0)),"")</f>
+        <f>IF($A31="","",IFERROR(INDEX($H$11:$H$20,MATCH($A31,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="G31" s="1" t="n"/>
-      <c r="H31" s="45" t="n">
-        <v>5</v>
+      <c r="H31" s="45">
+        <f>IF(COUNT($N$11:$N$20)&gt;=5,5,"")</f>
+        <v/>
       </c>
       <c r="I31" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($H31,$N$11:$N$20,0)),"")</f>
+        <f>IF($H31="","",IFERROR(INDEX($B$11:$B$20,MATCH($H31,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="J31" s="60" t="n"/>
       <c r="K31" s="60" t="n"/>
       <c r="L31" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($H31,$N$11:$N$20,0)),"")</f>
+        <f>IF($H31="","",IFERROR(INDEX($D$11:$D$20,MATCH($H31,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="M31" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($H31,$N$11:$N$20,0)),"")</f>
+        <f>IF($H31="","",IFERROR(INDEX($E$11:$E$20,MATCH($H31,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="N31" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($H31,$N$11:$N$20,0)),"")</f>
+        <f>IF($H31="","",IFERROR(INDEX($H$11:$H$20,MATCH($H31,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="O31" s="1" t="n"/>
     </row>
     <row r="32" ht="19" customHeight="1">
-      <c r="A32" s="45" t="n">
-        <v>6</v>
+      <c r="A32" s="45">
+        <f>IF(COUNT($M$11:$M$20)&gt;=6,6,"")</f>
+        <v/>
       </c>
       <c r="B32" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($A32,$M$11:$M$20,0)),"")</f>
+        <f>IF($A32="","",IFERROR(INDEX($B$11:$B$20,MATCH($A32,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="C32" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($A32,$M$11:$M$20,0)),"")</f>
+        <f>IF($A32="","",IFERROR(INDEX($D$11:$D$20,MATCH($A32,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="D32" s="60" t="n"/>
       <c r="E32" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($A32,$M$11:$M$20,0)),"")</f>
+        <f>IF($A32="","",IFERROR(INDEX($E$11:$E$20,MATCH($A32,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="F32" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($A32,$M$11:$M$20,0)),"")</f>
+        <f>IF($A32="","",IFERROR(INDEX($H$11:$H$20,MATCH($A32,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="G32" s="1" t="n"/>
-      <c r="H32" s="45" t="n">
-        <v>6</v>
+      <c r="H32" s="45">
+        <f>IF(COUNT($N$11:$N$20)&gt;=6,6,"")</f>
+        <v/>
       </c>
       <c r="I32" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($H32,$N$11:$N$20,0)),"")</f>
+        <f>IF($H32="","",IFERROR(INDEX($B$11:$B$20,MATCH($H32,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="J32" s="60" t="n"/>
       <c r="K32" s="60" t="n"/>
       <c r="L32" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($H32,$N$11:$N$20,0)),"")</f>
+        <f>IF($H32="","",IFERROR(INDEX($D$11:$D$20,MATCH($H32,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="M32" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($H32,$N$11:$N$20,0)),"")</f>
+        <f>IF($H32="","",IFERROR(INDEX($E$11:$E$20,MATCH($H32,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="N32" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($H32,$N$11:$N$20,0)),"")</f>
+        <f>IF($H32="","",IFERROR(INDEX($H$11:$H$20,MATCH($H32,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="O32" s="1" t="n"/>
     </row>
     <row r="33" ht="19" customHeight="1">
-      <c r="A33" s="45" t="n">
-        <v>7</v>
+      <c r="A33" s="45">
+        <f>IF(COUNT($M$11:$M$20)&gt;=7,7,"")</f>
+        <v/>
       </c>
       <c r="B33" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($A33,$M$11:$M$20,0)),"")</f>
+        <f>IF($A33="","",IFERROR(INDEX($B$11:$B$20,MATCH($A33,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="C33" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($A33,$M$11:$M$20,0)),"")</f>
+        <f>IF($A33="","",IFERROR(INDEX($D$11:$D$20,MATCH($A33,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="D33" s="60" t="n"/>
       <c r="E33" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($A33,$M$11:$M$20,0)),"")</f>
+        <f>IF($A33="","",IFERROR(INDEX($E$11:$E$20,MATCH($A33,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="F33" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($A33,$M$11:$M$20,0)),"")</f>
+        <f>IF($A33="","",IFERROR(INDEX($H$11:$H$20,MATCH($A33,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="G33" s="1" t="n"/>
-      <c r="H33" s="45" t="n">
-        <v>7</v>
+      <c r="H33" s="45">
+        <f>IF(COUNT($N$11:$N$20)&gt;=7,7,"")</f>
+        <v/>
       </c>
       <c r="I33" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($H33,$N$11:$N$20,0)),"")</f>
+        <f>IF($H33="","",IFERROR(INDEX($B$11:$B$20,MATCH($H33,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="J33" s="60" t="n"/>
       <c r="K33" s="60" t="n"/>
       <c r="L33" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($H33,$N$11:$N$20,0)),"")</f>
+        <f>IF($H33="","",IFERROR(INDEX($D$11:$D$20,MATCH($H33,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="M33" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($H33,$N$11:$N$20,0)),"")</f>
+        <f>IF($H33="","",IFERROR(INDEX($E$11:$E$20,MATCH($H33,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="N33" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($H33,$N$11:$N$20,0)),"")</f>
+        <f>IF($H33="","",IFERROR(INDEX($H$11:$H$20,MATCH($H33,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="O33" s="1" t="n"/>
     </row>
     <row r="34" ht="19" customHeight="1">
-      <c r="A34" s="45" t="n">
-        <v>8</v>
+      <c r="A34" s="45">
+        <f>IF(COUNT($M$11:$M$20)&gt;=8,8,"")</f>
+        <v/>
       </c>
       <c r="B34" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($A34,$M$11:$M$20,0)),"")</f>
+        <f>IF($A34="","",IFERROR(INDEX($B$11:$B$20,MATCH($A34,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="C34" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($A34,$M$11:$M$20,0)),"")</f>
+        <f>IF($A34="","",IFERROR(INDEX($D$11:$D$20,MATCH($A34,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="D34" s="60" t="n"/>
       <c r="E34" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($A34,$M$11:$M$20,0)),"")</f>
+        <f>IF($A34="","",IFERROR(INDEX($E$11:$E$20,MATCH($A34,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="F34" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($A34,$M$11:$M$20,0)),"")</f>
+        <f>IF($A34="","",IFERROR(INDEX($H$11:$H$20,MATCH($A34,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="G34" s="1" t="n"/>
-      <c r="H34" s="45" t="n">
-        <v>8</v>
+      <c r="H34" s="45">
+        <f>IF(COUNT($N$11:$N$20)&gt;=8,8,"")</f>
+        <v/>
       </c>
       <c r="I34" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($H34,$N$11:$N$20,0)),"")</f>
+        <f>IF($H34="","",IFERROR(INDEX($B$11:$B$20,MATCH($H34,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="J34" s="60" t="n"/>
       <c r="K34" s="60" t="n"/>
       <c r="L34" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($H34,$N$11:$N$20,0)),"")</f>
+        <f>IF($H34="","",IFERROR(INDEX($D$11:$D$20,MATCH($H34,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="M34" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($H34,$N$11:$N$20,0)),"")</f>
+        <f>IF($H34="","",IFERROR(INDEX($E$11:$E$20,MATCH($H34,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="N34" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($H34,$N$11:$N$20,0)),"")</f>
+        <f>IF($H34="","",IFERROR(INDEX($H$11:$H$20,MATCH($H34,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="O34" s="1" t="n"/>
     </row>
     <row r="35" ht="19" customHeight="1">
-      <c r="A35" s="45" t="n">
-        <v>9</v>
+      <c r="A35" s="45">
+        <f>IF(COUNT($M$11:$M$20)&gt;=9,9,"")</f>
+        <v/>
       </c>
       <c r="B35" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($A35,$M$11:$M$20,0)),"")</f>
+        <f>IF($A35="","",IFERROR(INDEX($B$11:$B$20,MATCH($A35,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="C35" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($A35,$M$11:$M$20,0)),"")</f>
+        <f>IF($A35="","",IFERROR(INDEX($D$11:$D$20,MATCH($A35,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="D35" s="60" t="n"/>
       <c r="E35" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($A35,$M$11:$M$20,0)),"")</f>
+        <f>IF($A35="","",IFERROR(INDEX($E$11:$E$20,MATCH($A35,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="F35" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($A35,$M$11:$M$20,0)),"")</f>
+        <f>IF($A35="","",IFERROR(INDEX($H$11:$H$20,MATCH($A35,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="G35" s="1" t="n"/>
-      <c r="H35" s="45" t="n">
-        <v>9</v>
+      <c r="H35" s="45">
+        <f>IF(COUNT($N$11:$N$20)&gt;=9,9,"")</f>
+        <v/>
       </c>
       <c r="I35" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($H35,$N$11:$N$20,0)),"")</f>
+        <f>IF($H35="","",IFERROR(INDEX($B$11:$B$20,MATCH($H35,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="J35" s="60" t="n"/>
       <c r="K35" s="60" t="n"/>
       <c r="L35" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($H35,$N$11:$N$20,0)),"")</f>
+        <f>IF($H35="","",IFERROR(INDEX($D$11:$D$20,MATCH($H35,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="M35" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($H35,$N$11:$N$20,0)),"")</f>
+        <f>IF($H35="","",IFERROR(INDEX($E$11:$E$20,MATCH($H35,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="N35" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($H35,$N$11:$N$20,0)),"")</f>
+        <f>IF($H35="","",IFERROR(INDEX($H$11:$H$20,MATCH($H35,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="O35" s="1" t="n"/>
     </row>
     <row r="36" ht="19" customHeight="1">
-      <c r="A36" s="45" t="n">
-        <v>10</v>
+      <c r="A36" s="45">
+        <f>IF(COUNT($M$11:$M$20)&gt;=10,10,"")</f>
+        <v/>
       </c>
       <c r="B36" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($A36,$M$11:$M$20,0)),"")</f>
+        <f>IF($A36="","",IFERROR(INDEX($B$11:$B$20,MATCH($A36,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="C36" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($A36,$M$11:$M$20,0)),"")</f>
+        <f>IF($A36="","",IFERROR(INDEX($D$11:$D$20,MATCH($A36,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="D36" s="60" t="n"/>
       <c r="E36" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($A36,$M$11:$M$20,0)),"")</f>
+        <f>IF($A36="","",IFERROR(INDEX($E$11:$E$20,MATCH($A36,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="F36" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($A36,$M$11:$M$20,0)),"")</f>
+        <f>IF($A36="","",IFERROR(INDEX($H$11:$H$20,MATCH($A36,$M$11:$M$20,0)),""))</f>
         <v/>
       </c>
       <c r="G36" s="1" t="n"/>
-      <c r="H36" s="45" t="n">
-        <v>10</v>
+      <c r="H36" s="45">
+        <f>IF(COUNT($N$11:$N$20)&gt;=10,10,"")</f>
+        <v/>
       </c>
       <c r="I36" s="37">
-        <f>IFERROR(INDEX($B$11:$B$20,MATCH($H36,$N$11:$N$20,0)),"")</f>
+        <f>IF($H36="","",IFERROR(INDEX($B$11:$B$20,MATCH($H36,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="J36" s="60" t="n"/>
       <c r="K36" s="60" t="n"/>
       <c r="L36" s="37">
-        <f>IFERROR(INDEX($D$11:$D$20,MATCH($H36,$N$11:$N$20,0)),"")</f>
+        <f>IF($H36="","",IFERROR(INDEX($D$11:$D$20,MATCH($H36,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="M36" s="61">
-        <f>IFERROR(INDEX($E$11:$E$20,MATCH($H36,$N$11:$N$20,0)),"")</f>
+        <f>IF($H36="","",IFERROR(INDEX($E$11:$E$20,MATCH($H36,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="N36" s="62">
-        <f>IFERROR(INDEX($H$11:$H$20,MATCH($H36,$N$11:$N$20,0)),"")</f>
+        <f>IF($H36="","",IFERROR(INDEX($H$11:$H$20,MATCH($H36,$N$11:$N$20,0)),""))</f>
         <v/>
       </c>
       <c r="O36" s="1" t="n"/>

</xml_diff>

<commit_message>
Trabalho em andamento dos agentes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LEmDYK8ehtpTRFSK7FMy6P
</commit_message>
<xml_diff>
--- a/produtos/chefoes-do-cartao/bonus/Placar-dos-Chefoes.xlsx
+++ b/produtos/chefoes-do-cartao/bonus/Placar-dos-Chefoes.xlsx
@@ -1255,7 +1255,7 @@
       </c>
       <c r="D7" s="1" t="n"/>
     </row>
-    <row r="8" ht="34" customHeight="1">
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="1" t="n"/>
       <c r="B8" s="7" t="inlineStr">
         <is>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="D8" s="1" t="n"/>
     </row>
-    <row r="9" ht="34" customHeight="1">
+    <row r="9" ht="48" customHeight="1">
       <c r="A9" s="1" t="n"/>
       <c r="B9" s="7" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="D9" s="1" t="n"/>
     </row>
-    <row r="10" ht="34" customHeight="1">
+    <row r="10" ht="48" customHeight="1">
       <c r="A10" s="1" t="n"/>
       <c r="B10" s="7" t="inlineStr">
         <is>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="D10" s="1" t="n"/>
     </row>
-    <row r="11" ht="34" customHeight="1">
+    <row r="11" ht="48" customHeight="1">
       <c r="A11" s="1" t="n"/>
       <c r="B11" s="7" t="inlineStr">
         <is>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="D11" s="1" t="n"/>
     </row>
-    <row r="12" ht="34" customHeight="1">
+    <row r="12" ht="48" customHeight="1">
       <c r="A12" s="1" t="n"/>
       <c r="B12" s="7" t="inlineStr">
         <is>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="D12" s="1" t="n"/>
     </row>
-    <row r="13" ht="34" customHeight="1">
+    <row r="13" ht="48" customHeight="1">
       <c r="A13" s="1" t="n"/>
       <c r="B13" s="7" t="inlineStr">
         <is>

</xml_diff>